<commit_message>
added cpi for 2025
</commit_message>
<xml_diff>
--- a/inputs/raw_index_data.xlsx
+++ b/inputs/raw_index_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleaw\Documents\PhD Fall 2021 - Spring 2022\Merriman RA\Fiscal Futures IGPA\Fiscal-Future-Topics\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F01543E-3208-44A9-AD56-D3C37D607D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D3A1721-9D90-4292-BBBF-A099BA0E01A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2922" yWindow="2688" windowWidth="17280" windowHeight="8994" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3366" windowWidth="17280" windowHeight="8994" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_fred_data" sheetId="1" r:id="rId1"/>
@@ -207,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -215,6 +215,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -883,8 +884,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="9.15625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
@@ -1575,6 +1579,18 @@
         <v>2024</v>
       </c>
       <c r="H28" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="5"/>
+      <c r="D29" s="2">
+        <v>317.67</v>
+      </c>
+      <c r="G29" s="2">
+        <v>2025</v>
+      </c>
+      <c r="H29" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>